<commit_message>
Final changes before release
</commit_message>
<xml_diff>
--- a/repairableExample/RawInputData/ComponentFailureData.xlsx
+++ b/repairableExample/RawInputData/ComponentFailureData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ttcd\Documents\MATLAB\PetriNetSimulate\repairableExample\RawInputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499B73DB-A588-413D-80A0-094B2D38779B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FBCB44-CDCF-49D0-A69D-9C2A69F5168B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$14</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Place Number</t>
   </si>
@@ -141,6 +141,15 @@
   </si>
   <si>
     <t>4,000 hours</t>
+  </si>
+  <si>
+    <t>PID</t>
+  </si>
+  <si>
+    <t>TransID</t>
+  </si>
+  <si>
+    <t>Repair</t>
   </si>
 </sst>
 </file>
@@ -663,24 +672,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.453125" customWidth="1"/>
     <col min="2" max="2" width="12.1796875" customWidth="1"/>
     <col min="3" max="3" width="67.453125" customWidth="1"/>
     <col min="4" max="4" width="24.453125" customWidth="1"/>
-    <col min="5" max="5" width="19.08984375" customWidth="1"/>
-    <col min="6" max="6" width="23.81640625" customWidth="1"/>
-    <col min="7" max="7" width="12.81640625" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="9.453125" customWidth="1"/>
-    <col min="10" max="10" width="11.08984375" customWidth="1"/>
-    <col min="12" max="12" width="22.54296875" customWidth="1"/>
-    <col min="13" max="13" width="2.7265625" customWidth="1"/>
+    <col min="5" max="8" width="19.08984375" customWidth="1"/>
+    <col min="9" max="9" width="23.81640625" customWidth="1"/>
+    <col min="10" max="10" width="12.81640625" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="9.453125" customWidth="1"/>
+    <col min="13" max="13" width="11.08984375" customWidth="1"/>
+    <col min="15" max="15" width="22.54296875" customWidth="1"/>
+    <col min="16" max="16" width="2.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -700,22 +709,31 @@
         <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -735,21 +753,30 @@
         <v>20</v>
       </c>
       <c r="G2" s="8">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8">
+        <v>1</v>
+      </c>
+      <c r="I2" s="8">
         <v>0</v>
       </c>
-      <c r="H2" s="10">
+      <c r="J2" s="8">
+        <v>0</v>
+      </c>
+      <c r="K2" s="10">
         <v>5000</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="O2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="9">
+      <c r="P2" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -769,39 +796,48 @@
         <v>21</v>
       </c>
       <c r="G3" s="8">
+        <v>2</v>
+      </c>
+      <c r="H3" s="8">
+        <v>2</v>
+      </c>
+      <c r="I3" s="8">
         <v>0</v>
       </c>
-      <c r="H3" s="10">
+      <c r="J3" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" s="10">
         <v>4000</v>
       </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="L3" s="9" t="s">
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="O3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M3" s="9">
+      <c r="P3" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="L4" s="9" t="s">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="O4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="9">
+      <c r="P4" s="9">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="L5" s="9" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="O5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="9">
+      <c r="P5" s="9">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J14" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J14">
+  <autoFilter ref="A1:M14" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M14">
       <sortCondition ref="A2:A14"/>
     </sortState>
   </autoFilter>

</xml_diff>